<commit_message>
Sparkline mini charts for agents without Code interpreter
- FSI Latest: last 12 quarters; WEO Data and GCC_Summary: 2010-2031;
  credit Latest: gap over the last 12 periods; each with its range
- Instructions: answer 'plot' requests with the sparkline table when
  Python is unavailable

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -503,18 +503,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,35 +532,45 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Gap mini chart, last 12 periods</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Gap mini chart range</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Credit-to-GDP ratio (% of GDP)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>HP trend (% of GDP)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Gap (pp of GDP)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gap a year earlier (pp)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Largest gap (pp)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Largest gap period</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
@@ -575,27 +587,37 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>▄██▆▄▄▆▃▁▃▄▅</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2014 to 2025: min -22.5, max 22.2</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>104.4</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>104</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>0.4</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>-6.2</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>22.2</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
@@ -612,27 +634,37 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>▄▅▇█▇▅▅▇▄▁▂▃</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2013 to 2024: min -12.8, max 17.1</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>73.7</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>-6.1</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>-8.699999999999999</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>17.1</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
@@ -649,27 +681,37 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>▂▄▅▄▃▅█▅▁▂▂▂</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2014 to 2025: min -5.7, max 45.4</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>125.3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>123.8</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>1.5</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>2.4</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>45.4</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
@@ -686,27 +728,37 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>▃▇▇▅▄▄█▄▁▂▃▅</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2014 to 2025: min -19.8, max 1.5</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>74.2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>82.7</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>-8.4</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>-13.4</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>1.5</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>

</xml_diff>

<commit_message>
Bank asset structure, stacked bar and pie charts, confidential bank-by-bank view
- Banking workbook: asset structure rows (BANK_STR_*, sum to 100%) and
  clearer nexus labels
- Agent chart(): kind='stack' draws stacked bars, new kind='pie' for one
  year; red CONFIDENTIAL label when the citation says so
- build_local_sources.py: HEAT_banks sheet (bank-by-bank, annual, with
  names) in the git-ignored local workbook
- Instructions 7,747 characters; tested end to end for Kuwait
- Stop tracking an accidental workbook copy; ignore '* - Copy*'

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latest" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit_GDP_Annual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Built on 2026-09-29 from the public IMF SDMX API (api.imf.org): dataset IMF.STA:MFS_DC (depository corporations survey) and IMF.RES:WEO (nominal GDP, domestic currency).</t>
+          <t>Built on 2026-09-30 from the public IMF SDMX API (api.imf.org): dataset IMF.STA:MFS_DC (depository corporations survey) and IMF.RES:WEO (nominal GDP, domestic currency).</t>
         </is>
       </c>
     </row>
@@ -488,7 +487,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>To refresh: run m365-agent/build_data_file.py from github.com/Aknarik/country-data and re-upload.</t>
+          <t>To refresh: run m365-agent/build_data_file.py and re-upload.</t>
         </is>
       </c>
     </row>
@@ -1154,6 +1153,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>83.00069999999999</v>
       </c>
@@ -1246,6 +1255,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
         <v>-16.4485</v>
       </c>
@@ -1460,6 +1479,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
         <v>76.1014</v>
       </c>
@@ -1552,6 +1581,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>-9.697100000000001</v>
       </c>
@@ -1716,6 +1755,7 @@
       <c r="AG8" t="n">
         <v>67.55589999999999</v>
       </c>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1763,6 +1803,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
         <v>37.5055</v>
       </c>
@@ -1805,6 +1855,7 @@
       <c r="AG9" t="n">
         <v>73.6733</v>
       </c>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1852,6 +1903,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>0.4929</v>
       </c>
@@ -1894,6 +1955,7 @@
       <c r="AG10" t="n">
         <v>-6.1174</v>
       </c>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2063,6 +2125,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
         <v>48.1645</v>
       </c>
@@ -2155,6 +2227,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
         <v>-8.4115</v>
       </c>
@@ -2199,1205 +2281,6 @@
       </c>
       <c r="AH13" t="n">
         <v>1.5407</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A189"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t># Country Data Assistant - tools for the Microsoft 365 Copilot agent's Code interpreter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t># build_data_file.py stores this file, one line per row, in a sheet "Code" of every workbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t># (and in Agent_tools.xlsx); the agent runs it with exec(). Keep it self-contained</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t># (pandas, numpy, matplotlib only).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>import glob, os, re, textwrap, numpy as np, pandas as pd, matplotlib.pyplot as plt</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>from matplotlib.ticker import MaxNLocator</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>fs = sorted({os.path.abspath(p) for pat in ('/mnt/**/*.xls*', '/home/**/*.xls*', '**/*.xls*')</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">             for p in glob.glob(pat, recursive=True)})</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>def xl(key, sheet):</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Load a sheet from the first workbook whose name contains `key`; None if not available."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    p = next((p for p in fs if key in os.path.basename(p)), None)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return pd.read_excel(p, sheet_name=sheet) if p else None</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>D, G = xl('World_Economic_Outlook', 'Data'), xl('World_Economic_Outlook', 'Groups')</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>F = xl('Financial_Soundness', 'FSI_Quarterly')</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>CQ, CA = xl('BIS_credit', 'Credit_GDP_Quarterly'), xl('BIS_credit', 'Credit_GDP_Annual')</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>M = xl('IMF_MFS_credit', 'Credit_GDP_Annual')</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>_loaded = {'D (IMF WEO)': D, 'G (groups)': G, 'F (FSI)': F, 'CQ/CA (BIS credit)': CQ, 'M (Gulf MFS credit)': M}</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>print('Loaded:', ', '.join(k for k, v in _loaded.items() if v is not None) or 'no data workbooks')</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>if any(v is None for v in _loaded.values()):</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    print('Not available:', ', '.join(k for k, v in _loaded.items() if v is None),</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">          '| workbooks found:', [os.path.basename(p) for p in fs])</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>BLUE, RED = '#4B82AD', '#c0392b'</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>PERIOD = re.compile(r'\d{4}(-Q\d)?')</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>def _style(ax):</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax.grid(alpha=0.3); ax.spines[['top', 'right']].set_visible(False)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>def _footer(fig, src):</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    fig.text(0.01, 0.01, textwrap.fill(src, 150), fontsize=8, color='dimgray')</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    fig.tight_layout(rect=(0, 0.06, 1, 1)); plt.show()</t>
-        </is>
-      </c>
-    </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t># --------------------------------------------------------------------------- charts</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>def chart(rows, start=2000, end=2031, kind='line', year=None):</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """kind='line' time series; 'bar' ranking for one period; 'gap' credit-to-GDP ratio + HP trend</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (top) and gap (bottom) - pass the 3 rows CREDIT_GDP, CREDIT_GDP_TREND, CREDIT_GDP_GAP."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    r0 = rows.iloc[-1]; P = int(r0['First projection year']) if 'First projection year' in rows else None</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    per = [c for c in rows.columns if PERIOD.fullmatch(str(c)) and start &lt;= int(str(c)[:4]) &lt;= end]</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    x = [int(c[:4]) + (int(c[-1]) - 1) / 4 if '-Q' in c else int(c) for c in per]</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce'); codes = list(rows['Indicator code'])</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    many = rows['Indicator'].nunique() &gt; 1; title = r0['Economy'] if many else r0['Indicator']</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    L = str(r0.get('Source link') or ''); src = f"Source: {r0['Citation']}. {L.rsplit('/', 1)[0] if '@' in L else L}"</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if kind == 'gap':</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        fig, (ax, a2) = plt.subplots(2, 1, figsize=(10, 7.5), sharex=True, gridspec_kw={'height_ratios': [2, 1]})</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        for c, lab, ls in (('CREDIT_GDP', 'Credit-to-GDP ratio', '-'), ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', '--')):</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            ax.plot(x, V.values[codes.index(c)], lw=2, ls=ls, label=lab)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        g = V.values[codes.index('CREDIT_GDP_GAP')]</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        a2.bar(x, g, width=0.22 if '-Q' in per[0] else 0.8, color=[RED if v &gt;= 0 else BLUE for v in g])</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        for h in (2, 10): a2.axhline(h, color='grey', ls=':', lw=1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        a2.axhline(0, color='black', lw=0.8); a2.set_ylabel('Gap, pp of GDP')</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        _style(a2); a2.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ax.set_ylabel('Percent of GDP'); ax.legend(frameon=False)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        title = f"{r0['Economy']}: credit-to-GDP ratio, trend and gap"</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    else:</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        fig, ax = plt.subplots(figsize=(10, 5.5))</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if kind == 'bar':</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        n = V.notna().sum(); y = str(year) if year else (str(P - 1) if P else n[n &gt;= 0.8 * n.max()].index[-1])</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        s = rows.set_index('Economy')[y].dropna().sort_values()</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ax.barh(s.index, s.values, color='#2a6fb0'); ax.set_xlabel(r0['Unit'])</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        title = f"{title}, {y}" + (' (IMF projection)' if P and int(y[:4]) &gt;= P else '')</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    elif kind == 'line':</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        for lab, v in zip(rows['Indicator'] if many else rows['Economy'], V.values):</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            ax.plot(x, v, lw=2, label=lab)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if V.min().min() &lt; 0 &lt; V.max().max(): ax.axhline(0, color='black', lw=0.8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if P and x[-1] &gt;= P:</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            ax.axvspan(P - 0.5, x[-1] + 0.5, color='grey', alpha=0.15, zorder=0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            ax.text(P, 0.98, ' IMF projections', transform=ax.get_xaxis_transform(), va='top', fontsize=9, color='dimgray')</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ax.set_ylabel(r0['Unit']); ax.legend(frameon=False); ax.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax.set_title(title, loc='left', weight='bold', color=BLUE); _style(ax)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    _footer(fig, src)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t># --------------------------------------------------------------------------- user data: credit gap</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>def hp_one_sided(y, lamb):</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """One-sided HP trend: for each t, fit a standard HP filter on y[0..t] and keep the last value."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    y = np.asarray(y, float); out = np.full(len(y), np.nan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    for t in range(1, len(y) + 1):</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if t &lt; 3:</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            out[t - 1] = y[t - 1]; continue</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        d = np.diff(np.eye(t), 2, axis=0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        out[t - 1] = np.linalg.solve(np.eye(t) + lamb * d.T @ d, y[:t])[-1]</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return out</t>
-        </is>
-      </c>
-    </row>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>def to_periods(index):</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Dates / 2020 / '2020Q1' / '2020-Q1' -&gt; '2020' or '2020-Q1'. Dates become quarters; a series</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    with only one date per year (e.g. every 31 Dec) becomes annual."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    out = []</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    for v in index:</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        s = str(v).strip().upper().replace(' ', '')</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if re.fullmatch(r'\d{4}(\.0)?', s): out.append(s[:4])</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        elif re.fullmatch(r'\d{4}-?Q[1-4]', s): out.append(f'{s[:4]}-Q{s[-1]}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        else: t = pd.Timestamp(v); out.append(f'{t.year}-Q{t.quarter}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if all('-Q' in p for p in out) and len({p[:4] for p in out}) == len(out):</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        out = [p[:4] for p in out]</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return out</t>
-        </is>
-      </c>
-    </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>def user_gap(credit=None, gdp=None, ratio=None, economy='User data', lamb=None, min_years=10, source='User-provided data'):</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Build the 3 gap rows from the user's own data, ready for chart(rows, kind='gap').</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Give either `ratio` (% of GDP) or `credit` and `gdp` as pandas Series indexed by period/date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Quarterly GDP is summed over the last 4 quarters (BIS method); annual GDP with quarterly credit</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    is matched by calendar year. lambda: 400,000 quarterly, 100,000 annual (override with lamb)."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if ratio is None:</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        c = pd.Series(credit.values, index=to_periods(credit.index), dtype=float).dropna()</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        g = pd.Series(gdp.values, index=to_periods(gdp.index), dtype=float).dropna()</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        qc, qg = '-Q' in c.index[0], '-Q' in g.index[0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if qc and qg: g = g.sort_index().rolling(4).sum()</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        elif qc: g = pd.Series(g.reindex([p[:4] for p in c.index]).values, index=c.index)</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ratio = 100 * c / g.reindex(c.index)</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    else:</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ratio = pd.Series(ratio.values, index=to_periods(ratio.index), dtype=float)</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    r = ratio.dropna().sort_index(); q = '-Q' in r.index[0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    lamb = lamb or (400_000 if q else 100_000)</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    tr = pd.Series(hp_one_sided(r.values, lamb), index=r.index)</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    tr.iloc[:min_years * (4 if q else 1)] = np.nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cite = f"{source}; trend and gap: own calculation, one-sided HP filter (lambda {lamb:,})"</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = [dict(Economy=economy, **{'Indicator code': k, 'Indicator': n, 'Unit': u, 'Citation': cite, 'Source link': ''}, **s.to_dict())</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            for k, n, u, s in (('CREDIT_GDP', 'Credit-to-GDP ratio', 'Percent of GDP', r),</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                               ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', 'Percent of GDP', tr),</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                               ('CREDIT_GDP_GAP', 'Credit-to-GDP gap', 'Percentage points of GDP', r - tr))]</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return pd.DataFrame(rows)</t>
-        </is>
-      </c>
-    </row>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t># --------------------------------------------------------------------------- FSI heat map</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t># Groups and directions come from the FSI workbook: column Group, and column "More vulnerable when"</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t># ("higher" or "lower"), set from a financial-sector vulnerability perspective.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>def percent_rank(s):</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Excel PERCENTRANK.INC of every value within its own series: (values below) / (n - 1)."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    s = s.dropna(); return (s.rank(method='min') - 1) / (len(s) - 1) if len(s) &gt; 1 else s * np.nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>def fsi_heatmap(country, quarters=12, min_history=8):</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Heat map of FSIs: colour = vulnerability percentile vs the country's own history</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (0 = least vulnerable ever, dark blue; 1 = most vulnerable ever, dark red); cells show actual values."""</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = F[(F['Economy'].str.lower() == country.lower()) | (F['Economy code'] == country.upper())]</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = rows.drop_duplicates('Indicator code').set_index('Indicator code')</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    per = [c for c in rows.columns if re.fullmatch(r'\d{4}-Q\d', str(c))]</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce')</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V = V[V.notna().sum(axis=1) &gt;= min_history]</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = rows.loc[V.index]</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    R = V.apply(percent_rank, axis=1).reindex(columns=per)</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    lower = (rows['More vulnerable when'] == 'lower').values; R.loc[lower] = 1 - R.loc[lower]</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    first = min(V.apply(lambda r: r.first_valid_index(), axis=1).dropna())</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cols = [c for c in per if V[c].notna().any()][-quarters:]</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V, R = V[cols], R[cols]</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    # explicit layout in inches: labels left, group names right, colour bar and source below</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    L = 0.3 + 0.062 * rows['Indicator'].str.len().max(); Rt = 0.4 + 0.07 * rows['Group'].str.len().max()</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    w, h, top, bot = 0.7 * len(cols), 0.42 * len(V), 0.75, 1.75</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    W, H = L + w + Rt, top + h + bot</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    fig = plt.figure(figsize=(W, H)); ax = fig.add_axes([L / W, bot / H, w / W, h / H])</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    im = ax.imshow(R.values.astype(float), cmap='RdBu_r', vmin=0, vmax=1, aspect='auto')</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    for i in range(len(V)):</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        for j in range(len(cols)):</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            v, r = V.iat[i, j], R.iat[i, j]</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            if pd.notna(v):</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                ax.text(j, i, f'{v:.1f}', ha='center', va='center', fontsize=8,</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                        color='white' if pd.notna(r) and abs(r - 0.5) &gt; 0.3 else 'black')</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax.set_yticks(range(len(V))); ax.set_yticklabels(rows['Indicator'], fontsize=8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax.set_xticks(range(len(cols))); ax.set_xticklabels(cols, rotation=45, ha='right', fontsize=8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    groups = list(rows['Group'])</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    starts = [i for i in range(len(groups)) if i == 0 or groups[i] != groups[i - 1]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    for i in starts[1:]: ax.axhline(i - 0.5, color='black', lw=1.2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax2 = ax.twinx(); ax2.set_ylim(ax.get_ylim())</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax2.set_yticks([(s + e - 1) / 2 for s, e in zip(starts, starts[1:] + [len(groups)])])</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax2.set_yticklabels([groups[s] for s in starts], fontsize=8, weight='bold', color=BLUE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax2.tick_params(length=0); ax2.spines[:].set_visible(False)</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cax = fig.add_axes([L / W, 0.55 / H, min(w, 5) / W, 0.13 / H])</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cb = fig.colorbar(im, cax=cax, orientation='horizontal'); cb.set_ticks([0, 0.5, 1])</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cb.set_ticklabels(['Less vulnerable', 'Median', 'More vulnerable']); cb.ax.tick_params(labelsize=8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ax.set_title(f"{rows['Economy'].dropna().iloc[0]}: financial soundness heat map\n"</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                 "colour = percent rank vs own history (dark red = most vulnerable, dark blue = least)",</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                 loc='left', weight='bold', color=BLUE, fontsize=10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    note = f"Each indicator is ranked against all its own quarters since {first} (Excel PERCENTRANK.INC)."</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    fig.text(0.01, 0.06 / H, textwrap.fill(f"Source: {rows['Citation'].dropna().iloc[0]}. {note}", int(W * 14)),</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">             fontsize=8, color='dimgray'); plt.show()</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return pd.DataFrame({'Group': rows['Group'].values, 'Indicator': rows['Indicator'].values,</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                         'Latest value': V.ffill(axis=1).iloc[:, -1].round(2).values,</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                         'Vulnerability percentile': R.ffill(axis=1).iloc[:, -1].round(2).values})</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agents: 'Country: Indicator' titles, forecast axis, iMaPP note, gap data-length guidance
- Titles read 'Kuwait: Real GDP growth' / 'GCC: ...' (group detected); capital after the colon
- Forecast charts end at the shaded projection area
- Gap chart note explains how net tightening/loosening is counted (iMaPP +1/-1 per tool-month)
- MFS credit workbook README: recommended data length for user gaps (20+ years, minimum 10),
  quoting Drehmann & Tsatsaronis (2014), BCBS (2010), ESRB/2014/1, Ravn & Uhlig (2002)
- user_gap warns under 20 years and stops under 10

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -48,8 +48,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -488,6 +491,55 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>To refresh: run m365-agent/build_data_file.py and re-upload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>USER-BUILT GAPS: RECOMMENDED DATA LENGTH. Use at least 20 years (80 quarters) of credit-to-GDP data where possible, and never less than 10 years. The first 10 years only start the one-sided HP trend and are not reported, so with 10-20 years of data the gap covers fewer than 10 years and should be read with caution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Why: Drehmann and Tsatsaronis (2014, p. 14 of the article PDF) 'validate the practical rule of thumb that suggests using the credit gap only when at least 10 years of data for the credit-to-GDP ratio are already available', but note that at the start of a series 'it can take 20 years for measurement differences to fully disappear' (p. 13) and that 'we need at least 20 years of data in order to properly assess the forecasting ability of the credit gap' (p. 10). Credit cycles are 'on average about four times longer than standard business cycles and crises tend to occur once every 20-25 years' (p. 12).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Structural breaks: adjust the credit series for breaks first; after a large break 'it takes more than 20 years for such an effect of this magnitude to fully disappear' (Drehmann and Tsatsaronis, 2014, p. 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Quarterly data (preferred): ratio = credit at end of quarter / sum of GDP over the last 4 quarters x 100; one-sided HP trend with lambda 400,000 (BCBS, 2010, Annex 1; ESRB Recommendation ESRB/2014/1, Annex, Part II).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Oil exporters: a ratio to non-oil GDP (user data) avoids oil-price swings in GDP; say that the GDP measure is user data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>References: BCBS (2010), Guidance for national authorities operating the countercyclical capital buffer, Basel Committee on Banking Supervision, December, https://www.bis.org/publ/bcbs187.htm. Drehmann, M. and K. Tsatsaronis (2014), 'The credit-to-GDP gap and countercyclical capital buffers: questions and answers', BIS Quarterly Review, March, https://www.bis.org/publ/qtrpdf/r_qt1403g.htm. ESRB (2014), Recommendation of the European Systemic Risk Board on guidance for setting countercyclical buffer rates (ESRB/2014/1), OJ C 293, 2.9.2014, https://www.esrb.europa.eu/pub/pdf/recommendations/140630_ESRB_Recommendation.en.pdf. Ravn, M. and H. Uhlig (2002), 'On adjusting the Hodrick-Prescott filter for the frequency of observations', Review of Economics and Statistics 84(2).</t>
         </is>
       </c>
     </row>
@@ -1153,16 +1205,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>83.00069999999999</v>
       </c>
@@ -1255,16 +1297,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
         <v>-16.4485</v>
       </c>
@@ -1479,16 +1511,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
         <v>76.1014</v>
       </c>
@@ -1581,16 +1603,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>-9.697100000000001</v>
       </c>
@@ -1755,7 +1767,6 @@
       <c r="AG8" t="n">
         <v>67.55589999999999</v>
       </c>
-      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1803,16 +1814,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
         <v>37.5055</v>
       </c>
@@ -1855,7 +1856,6 @@
       <c r="AG9" t="n">
         <v>73.6733</v>
       </c>
-      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1903,16 +1903,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>0.4929</v>
       </c>
@@ -1955,7 +1945,6 @@
       <c r="AG10" t="n">
         <v>-6.1174</v>
       </c>
-      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2125,16 +2114,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
         <v>48.1645</v>
       </c>
@@ -2227,16 +2206,6 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
         <v>-8.4115</v>
       </c>

</xml_diff>

<commit_message>
Charts: 'percent' instead of '%', last values labelled, grey band for projections, legends below
- Data labels in all workbooks use 'percent' (write_book converts Indicator/Unit on every build)
- Latest observation printed at the end of each line (and last actual bar in the WEO dashboard)
- Projections shown only by grey shading (no projection wording in titles)
- Legends placed under the charts

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -1060,7 +1060,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), % of GDP</t>
+          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), % of GDP</t>
+          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), % of GDP</t>
+          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), % of GDP</t>
+          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>

<commit_message>
Fix Gulf MFS credit measure: keep claims on public NFCs (Kuwait series break)
Kuwait reports claims on public non-financial corporations only from 2020 (zero
before), so subtracting them cut credit by ~7-8 pp of GDP from 2020 and biased
the gap down (2025: 0.4 pp -> 2.7 pp after the fix). Credit is now depository
corporations' claims on other sectors for all four Gulf countries, consistent over
time and in line with the BIS PNFS definition (NFCs include public corporations).
SAMA step falls back to the last downloaded bulletin when the site is unreachable.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -48,11 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +445,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors minus claims on public non-financial corporations, end of year, domestic currency. The narrower 'claims on private sector' series is not used because it has a reclassification break for Kuwait.</t>
+          <t>Credit = depository corporations' claims on other sectors, end of year, domestic currency. Claims on public non-financial corporations are included, as in the BIS definition of credit to the private non-financial sector (which covers publicly owned corporations), and because Kuwait reports them separately only from 2020 (zero before), so subtracting them would break the series. The narrower 'claims on private sector' series is not used because it has a reclassification break for Kuwait.</t>
         </is>
       </c>
     </row>
@@ -483,63 +480,63 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cite the 'Citation' column (IMF; trend and gap are own calculations), not this workbook.</t>
+          <t>USER-BUILT GAPS: RECOMMENDED DATA LENGTH. Use at least 20 years (80 quarters) of credit-to-GDP data where possible, and never less than 10 years. The first 10 years only start the one-sided HP trend and are not reported, so with 10-20 years of data the gap covers fewer than 10 years and should be read with caution.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Why: Drehmann and Tsatsaronis (2014, p. 14 of the article PDF) 'validate the practical rule of thumb that suggests using the credit gap only when at least 10 years of data for the credit-to-GDP ratio are already available', but note that at the start of a series 'it can take 20 years for measurement differences to fully disappear' (p. 13) and that 'we need at least 20 years of data in order to properly assess the forecasting ability of the credit gap' (p. 10). Credit cycles are 'on average about four times longer than standard business cycles and crises tend to occur once every 20-25 years' (p. 12).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Structural breaks: adjust the credit series for breaks first; after a large break 'it takes more than 20 years for such an effect of this magnitude to fully disappear' (Drehmann and Tsatsaronis, 2014, p. 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Quarterly data (preferred): ratio = credit at end of quarter / sum of GDP over the last 4 quarters x 100; one-sided HP trend with lambda 400,000 (BCBS, 2010, Annex 1; ESRB Recommendation ESRB/2014/1, Annex, Part II).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Oil exporters: a ratio to non-oil GDP (user data) avoids oil-price swings in GDP; say that the GDP measure is user data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>References: BCBS (2010), Guidance for national authorities operating the countercyclical capital buffer, Basel Committee on Banking Supervision, December, https://www.bis.org/publ/bcbs187.htm. Drehmann, M. and K. Tsatsaronis (2014), 'The credit-to-GDP gap and countercyclical capital buffers: questions and answers', BIS Quarterly Review, March, https://www.bis.org/publ/qtrpdf/r_qt1403g.htm. ESRB (2014), Recommendation of the European Systemic Risk Board on guidance for setting countercyclical buffer rates (ESRB/2014/1), OJ C 293, 2.9.2014, https://www.esrb.europa.eu/pub/pdf/recommendations/140630_ESRB_Recommendation.en.pdf. Ravn, M. and H. Uhlig (2002), 'On adjusting the Hodrick-Prescott filter for the frequency of observations', Review of Economics and Statistics 84(2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cite the 'Citation' column (IMF; trend and gap are own calculations), not this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>To refresh: run m365-agent/build_data_file.py and re-upload.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>USER-BUILT GAPS: RECOMMENDED DATA LENGTH. Use at least 20 years (80 quarters) of credit-to-GDP data where possible, and never less than 10 years. The first 10 years only start the one-sided HP trend and are not reported, so with 10-20 years of data the gap covers fewer than 10 years and should be read with caution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Why: Drehmann and Tsatsaronis (2014, p. 14 of the article PDF) 'validate the practical rule of thumb that suggests using the credit gap only when at least 10 years of data for the credit-to-GDP ratio are already available', but note that at the start of a series 'it can take 20 years for measurement differences to fully disappear' (p. 13) and that 'we need at least 20 years of data in order to properly assess the forecasting ability of the credit gap' (p. 10). Credit cycles are 'on average about four times longer than standard business cycles and crises tend to occur once every 20-25 years' (p. 12).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Structural breaks: adjust the credit series for breaks first; after a large break 'it takes more than 20 years for such an effect of this magnitude to fully disappear' (Drehmann and Tsatsaronis, 2014, p. 15).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Quarterly data (preferred): ratio = credit at end of quarter / sum of GDP over the last 4 quarters x 100; one-sided HP trend with lambda 400,000 (BCBS, 2010, Annex 1; ESRB Recommendation ESRB/2014/1, Annex, Part II).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Oil exporters: a ratio to non-oil GDP (user data) avoids oil-price swings in GDP; say that the GDP measure is user data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>References: BCBS (2010), Guidance for national authorities operating the countercyclical capital buffer, Basel Committee on Banking Supervision, December, https://www.bis.org/publ/bcbs187.htm. Drehmann, M. and K. Tsatsaronis (2014), 'The credit-to-GDP gap and countercyclical capital buffers: questions and answers', BIS Quarterly Review, March, https://www.bis.org/publ/qtrpdf/r_qt1403g.htm. ESRB (2014), Recommendation of the European Systemic Risk Board on guidance for setting countercyclical buffer rates (ESRB/2014/1), OJ C 293, 2.9.2014, https://www.esrb.europa.eu/pub/pdf/recommendations/140630_ESRB_Recommendation.en.pdf. Ravn, M. and H. Uhlig (2002), 'On adjusting the Hodrick-Prescott filter for the frequency of observations', Review of Economics and Statistics 84(2).</t>
         </is>
       </c>
     </row>
@@ -640,25 +637,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>▄██▆▄▄▆▃▁▃▄▅</t>
+          <t>▄██▆▄▄▇▃▁▃▄▅</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -22.5, max 22.2</t>
+          <t>2014 to 2025: min -19.7, max 22.2</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>104.4</v>
+        <v>112.6</v>
       </c>
       <c r="F2" t="n">
-        <v>104</v>
+        <v>109.8</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4</v>
+        <v>2.7</v>
       </c>
       <c r="H2" t="n">
-        <v>-6.2</v>
+        <v>-4.1</v>
       </c>
       <c r="I2" t="n">
         <v>22.2</v>
@@ -670,7 +667,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
     </row>
@@ -692,23 +689,23 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2013 to 2024: min -12.8, max 17.1</t>
+          <t>2013 to 2024: min -13.7, max 17.6</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>67.59999999999999</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>73.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>-6.1</v>
+        <v>-6</v>
       </c>
       <c r="H3" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.9</v>
       </c>
       <c r="I3" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -717,7 +714,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
     </row>
@@ -734,28 +731,28 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>▂▄▅▄▃▅█▅▁▂▂▂</t>
+          <t>▂▅▅▄▃▄█▅▁▂▂▂</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -5.7, max 45.4</t>
+          <t>2014 to 2025: min -12.6, max 51.5</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>125.3</v>
+        <v>160.1</v>
       </c>
       <c r="F4" t="n">
-        <v>123.8</v>
+        <v>163.5</v>
       </c>
       <c r="G4" t="n">
-        <v>1.5</v>
+        <v>-3.4</v>
       </c>
       <c r="H4" t="n">
-        <v>2.4</v>
+        <v>-1.6</v>
       </c>
       <c r="I4" t="n">
-        <v>45.4</v>
+        <v>51.5</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -764,7 +761,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
     </row>
@@ -781,28 +778,28 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>▃▇▇▅▄▄█▄▁▂▃▅</t>
+          <t>▄▇▇▅▄▄█▄▁▂▃▄</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -19.8, max 1.5</t>
+          <t>2014 to 2025: min -22.9, max 4.2</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>74.2</v>
+        <v>91.2</v>
       </c>
       <c r="F5" t="n">
-        <v>82.7</v>
+        <v>102.2</v>
       </c>
       <c r="G5" t="n">
-        <v>-8.4</v>
+        <v>-11</v>
       </c>
       <c r="H5" t="n">
-        <v>-13.4</v>
+        <v>-16.1</v>
       </c>
       <c r="I5" t="n">
-        <v>1.5</v>
+        <v>4.2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -811,7 +808,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
     </row>
@@ -857,10 +854,10 @@
     <col width="9" customWidth="1" min="26" max="26"/>
     <col width="9" customWidth="1" min="27" max="27"/>
     <col width="9" customWidth="1" min="28" max="28"/>
-    <col width="9" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
     <col width="10" customWidth="1" min="30" max="30"/>
     <col width="10" customWidth="1" min="31" max="31"/>
-    <col width="9" customWidth="1" min="32" max="32"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
     <col width="10" customWidth="1" min="33" max="33"/>
     <col width="10" customWidth="1" min="34" max="34"/>
   </cols>
@@ -1060,7 +1057,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
+          <t>Credit to the non-government sector (claims on other sectors), percent of GDP</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1070,12 +1067,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1084,79 +1081,79 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>35.3159</v>
+        <v>36.7017</v>
       </c>
       <c r="K2" t="n">
-        <v>37.031</v>
+        <v>38.7969</v>
       </c>
       <c r="L2" t="n">
-        <v>37.1103</v>
+        <v>39.9549</v>
       </c>
       <c r="M2" t="n">
-        <v>38.9448</v>
+        <v>41.5024</v>
       </c>
       <c r="N2" t="n">
-        <v>46.0636</v>
+        <v>49.8019</v>
       </c>
       <c r="O2" t="n">
-        <v>51.2614</v>
+        <v>55.3071</v>
       </c>
       <c r="P2" t="n">
-        <v>61.8745</v>
+        <v>66.6666</v>
       </c>
       <c r="Q2" t="n">
-        <v>75.6741</v>
+        <v>80.90940000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>94.2923</v>
+        <v>102.5895</v>
       </c>
       <c r="S2" t="n">
-        <v>78.1528</v>
+        <v>85.90219999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>66.5522</v>
+        <v>75.39919999999999</v>
       </c>
       <c r="U2" t="n">
-        <v>63.833</v>
+        <v>73.0497</v>
       </c>
       <c r="V2" t="n">
-        <v>63.2753</v>
+        <v>75.11109999999999</v>
       </c>
       <c r="W2" t="n">
-        <v>64.16849999999999</v>
+        <v>76.7752</v>
       </c>
       <c r="X2" t="n">
-        <v>77.6568</v>
+        <v>92.2623</v>
       </c>
       <c r="Y2" t="n">
-        <v>80.5989</v>
+        <v>96.63</v>
       </c>
       <c r="Z2" t="n">
-        <v>76.90009999999999</v>
+        <v>91.2307</v>
       </c>
       <c r="AA2" t="n">
-        <v>73.1746</v>
+        <v>86.107</v>
       </c>
       <c r="AB2" t="n">
-        <v>74.3584</v>
+        <v>88.3907</v>
       </c>
       <c r="AC2" t="n">
-        <v>88.1795</v>
+        <v>108.1365</v>
       </c>
       <c r="AD2" t="n">
-        <v>75.5707</v>
+        <v>93.4845</v>
       </c>
       <c r="AE2" t="n">
-        <v>64.92149999999999</v>
+        <v>80.20480000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>67.64700000000001</v>
+        <v>84.8776</v>
       </c>
       <c r="AG2" t="n">
-        <v>69.24769999999999</v>
+        <v>85.7444</v>
       </c>
       <c r="AH2" t="n">
-        <v>74.2201</v>
+        <v>91.2216</v>
       </c>
     </row>
     <row r="3">
@@ -1192,12 +1189,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1205,50 +1202,60 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>83.00069999999999</v>
+        <v>91.47920000000001</v>
       </c>
       <c r="U3" t="n">
-        <v>81.0732</v>
+        <v>90.30800000000001</v>
       </c>
       <c r="V3" t="n">
-        <v>79.33110000000001</v>
+        <v>89.8339</v>
       </c>
       <c r="W3" t="n">
-        <v>78.1123</v>
+        <v>89.7681</v>
       </c>
       <c r="X3" t="n">
-        <v>80.3329</v>
+        <v>93.35429999999999</v>
       </c>
       <c r="Y3" t="n">
-        <v>82.6981</v>
+        <v>97.11069999999999</v>
       </c>
       <c r="Z3" t="n">
-        <v>83.7392</v>
+        <v>98.886</v>
       </c>
       <c r="AA3" t="n">
-        <v>83.76130000000001</v>
+        <v>99.20010000000001</v>
       </c>
       <c r="AB3" t="n">
-        <v>83.9521</v>
+        <v>99.8267</v>
       </c>
       <c r="AC3" t="n">
-        <v>86.63379999999999</v>
+        <v>103.9576</v>
       </c>
       <c r="AD3" t="n">
-        <v>86.5985</v>
+        <v>104.7614</v>
       </c>
       <c r="AE3" t="n">
-        <v>84.7038</v>
+        <v>103.1124</v>
       </c>
       <c r="AF3" t="n">
-        <v>83.488</v>
+        <v>102.4087</v>
       </c>
       <c r="AG3" t="n">
-        <v>82.6574</v>
+        <v>101.8875</v>
       </c>
       <c r="AH3" t="n">
-        <v>82.6617</v>
+        <v>102.2213</v>
       </c>
     </row>
     <row r="4">
@@ -1284,12 +1291,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1297,50 +1304,60 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>-16.4485</v>
+        <v>-16.08</v>
       </c>
       <c r="U4" t="n">
-        <v>-17.2402</v>
+        <v>-17.2583</v>
       </c>
       <c r="V4" t="n">
-        <v>-16.0557</v>
+        <v>-14.7228</v>
       </c>
       <c r="W4" t="n">
-        <v>-13.9438</v>
+        <v>-12.9929</v>
       </c>
       <c r="X4" t="n">
-        <v>-2.6761</v>
+        <v>-1.092</v>
       </c>
       <c r="Y4" t="n">
-        <v>-2.0991</v>
+        <v>-0.4806</v>
       </c>
       <c r="Z4" t="n">
-        <v>-6.839</v>
+        <v>-7.6553</v>
       </c>
       <c r="AA4" t="n">
-        <v>-10.5867</v>
+        <v>-13.0931</v>
       </c>
       <c r="AB4" t="n">
-        <v>-9.5937</v>
+        <v>-11.436</v>
       </c>
       <c r="AC4" t="n">
-        <v>1.5457</v>
+        <v>4.1788</v>
       </c>
       <c r="AD4" t="n">
-        <v>-11.0278</v>
+        <v>-11.277</v>
       </c>
       <c r="AE4" t="n">
-        <v>-19.7824</v>
+        <v>-22.9076</v>
       </c>
       <c r="AF4" t="n">
-        <v>-15.841</v>
+        <v>-17.5311</v>
       </c>
       <c r="AG4" t="n">
-        <v>-13.4097</v>
+        <v>-16.1431</v>
       </c>
       <c r="AH4" t="n">
-        <v>-8.441599999999999</v>
+        <v>-10.9997</v>
       </c>
     </row>
     <row r="5">
@@ -1366,7 +1383,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
+          <t>Credit to the non-government sector (claims on other sectors), percent of GDP</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1376,12 +1393,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1447,22 +1464,22 @@
         <v>94.7747</v>
       </c>
       <c r="AC5" t="n">
-        <v>114.1506</v>
+        <v>122.7509</v>
       </c>
       <c r="AD5" t="n">
-        <v>91.30629999999999</v>
+        <v>99.1533</v>
       </c>
       <c r="AE5" t="n">
-        <v>78.4889</v>
+        <v>84.8875</v>
       </c>
       <c r="AF5" t="n">
-        <v>88.9264</v>
+        <v>96.1699</v>
       </c>
       <c r="AG5" t="n">
-        <v>95.74169999999999</v>
+        <v>102.8322</v>
       </c>
       <c r="AH5" t="n">
-        <v>104.4037</v>
+        <v>112.559</v>
       </c>
     </row>
     <row r="6">
@@ -1498,12 +1515,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1511,6 +1528,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
         <v>76.1014</v>
       </c>
@@ -1539,22 +1566,22 @@
         <v>97.4653</v>
       </c>
       <c r="AC6" t="n">
-        <v>102.6938</v>
+        <v>104.2959</v>
       </c>
       <c r="AD6" t="n">
-        <v>102.9737</v>
+        <v>105.7906</v>
       </c>
       <c r="AE6" t="n">
-        <v>100.9675</v>
+        <v>104.566</v>
       </c>
       <c r="AF6" t="n">
-        <v>100.912</v>
+        <v>105.3136</v>
       </c>
       <c r="AG6" t="n">
-        <v>101.8955</v>
+        <v>106.96</v>
       </c>
       <c r="AH6" t="n">
-        <v>104.0242</v>
+        <v>109.8197</v>
       </c>
     </row>
     <row r="7">
@@ -1590,12 +1617,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1603,6 +1630,16 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>-9.697100000000001</v>
       </c>
@@ -1631,22 +1668,22 @@
         <v>-2.6906</v>
       </c>
       <c r="AC7" t="n">
-        <v>11.4568</v>
+        <v>18.4549</v>
       </c>
       <c r="AD7" t="n">
-        <v>-11.6674</v>
+        <v>-6.6373</v>
       </c>
       <c r="AE7" t="n">
-        <v>-22.4785</v>
+        <v>-19.6785</v>
       </c>
       <c r="AF7" t="n">
-        <v>-11.9856</v>
+        <v>-9.143599999999999</v>
       </c>
       <c r="AG7" t="n">
-        <v>-6.1538</v>
+        <v>-4.1278</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.3795</v>
+        <v>2.7393</v>
       </c>
     </row>
     <row r="8">
@@ -1672,7 +1709,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
+          <t>Credit to the non-government sector (claims on other sectors), percent of GDP</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1682,12 +1719,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1696,77 +1733,78 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>35.1537</v>
+        <v>35.4823</v>
       </c>
       <c r="K8" t="n">
-        <v>33.9703</v>
+        <v>34.489</v>
       </c>
       <c r="L8" t="n">
-        <v>32.1771</v>
+        <v>32.9028</v>
       </c>
       <c r="M8" t="n">
-        <v>29.8652</v>
+        <v>30.6655</v>
       </c>
       <c r="N8" t="n">
-        <v>26.8302</v>
+        <v>27.6494</v>
       </c>
       <c r="O8" t="n">
-        <v>26.8602</v>
+        <v>28.056</v>
       </c>
       <c r="P8" t="n">
-        <v>32.6715</v>
+        <v>34.6356</v>
       </c>
       <c r="Q8" t="n">
-        <v>32.4587</v>
+        <v>34.2065</v>
       </c>
       <c r="R8" t="n">
-        <v>42.9384</v>
+        <v>45.6472</v>
       </c>
       <c r="S8" t="n">
-        <v>40.2649</v>
+        <v>44.0152</v>
       </c>
       <c r="T8" t="n">
-        <v>37.9984</v>
+        <v>42.936</v>
       </c>
       <c r="U8" t="n">
-        <v>38.8356</v>
+        <v>43.9361</v>
       </c>
       <c r="V8" t="n">
-        <v>40.7373</v>
+        <v>45.7979</v>
       </c>
       <c r="W8" t="n">
-        <v>43.7281</v>
+        <v>49.3844</v>
       </c>
       <c r="X8" t="n">
-        <v>61.4059</v>
+        <v>67.9558</v>
       </c>
       <c r="Y8" t="n">
-        <v>70.3506</v>
+        <v>77.6144</v>
       </c>
       <c r="Z8" t="n">
-        <v>69.3703</v>
+        <v>76.8934</v>
       </c>
       <c r="AA8" t="n">
-        <v>64.67789999999999</v>
+        <v>72.2483</v>
       </c>
       <c r="AB8" t="n">
-        <v>68.9603</v>
+        <v>77.0073</v>
       </c>
       <c r="AC8" t="n">
-        <v>80.7657</v>
+        <v>91.5299</v>
       </c>
       <c r="AD8" t="n">
-        <v>72.0866</v>
+        <v>83.262</v>
       </c>
       <c r="AE8" t="n">
-        <v>59.1967</v>
+        <v>68.45269999999999</v>
       </c>
       <c r="AF8" t="n">
-        <v>63.8467</v>
+        <v>74.4177</v>
       </c>
       <c r="AG8" t="n">
-        <v>67.55589999999999</v>
-      </c>
+        <v>78.86320000000001</v>
+      </c>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1801,12 +1839,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1814,48 +1852,59 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>37.5055</v>
+        <v>41.3218</v>
       </c>
       <c r="U9" t="n">
-        <v>38.4284</v>
+        <v>42.9118</v>
       </c>
       <c r="V9" t="n">
-        <v>39.6249</v>
+        <v>44.5879</v>
       </c>
       <c r="W9" t="n">
-        <v>41.2938</v>
+        <v>46.7672</v>
       </c>
       <c r="X9" t="n">
-        <v>46.8557</v>
+        <v>52.9337</v>
       </c>
       <c r="Y9" t="n">
-        <v>53.2989</v>
+        <v>60.01</v>
       </c>
       <c r="Z9" t="n">
-        <v>58.2529</v>
+        <v>65.5201</v>
       </c>
       <c r="AA9" t="n">
-        <v>61.2959</v>
+        <v>69.0164</v>
       </c>
       <c r="AB9" t="n">
-        <v>64.59950000000001</v>
+        <v>72.777</v>
       </c>
       <c r="AC9" t="n">
-        <v>69.5087</v>
+        <v>78.5637</v>
       </c>
       <c r="AD9" t="n">
-        <v>72.04900000000001</v>
+        <v>81.9062</v>
       </c>
       <c r="AE9" t="n">
-        <v>71.95489999999999</v>
+        <v>82.15519999999999</v>
       </c>
       <c r="AF9" t="n">
-        <v>72.5878</v>
+        <v>83.2869</v>
       </c>
       <c r="AG9" t="n">
-        <v>73.6733</v>
-      </c>
+        <v>84.9081</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1890,12 +1939,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1903,48 +1952,59 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
-        <v>0.4929</v>
+        <v>1.6141</v>
       </c>
       <c r="U10" t="n">
-        <v>0.4071</v>
+        <v>1.0243</v>
       </c>
       <c r="V10" t="n">
-        <v>1.1124</v>
+        <v>1.21</v>
       </c>
       <c r="W10" t="n">
-        <v>2.4343</v>
+        <v>2.6172</v>
       </c>
       <c r="X10" t="n">
-        <v>14.5502</v>
+        <v>15.0221</v>
       </c>
       <c r="Y10" t="n">
-        <v>17.0517</v>
+        <v>17.6044</v>
       </c>
       <c r="Z10" t="n">
-        <v>11.1174</v>
+        <v>11.3732</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.382</v>
+        <v>3.2319</v>
       </c>
       <c r="AB10" t="n">
-        <v>4.3608</v>
+        <v>4.2303</v>
       </c>
       <c r="AC10" t="n">
-        <v>11.257</v>
+        <v>12.9662</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.0376</v>
+        <v>1.3559</v>
       </c>
       <c r="AE10" t="n">
-        <v>-12.7582</v>
+        <v>-13.7025</v>
       </c>
       <c r="AF10" t="n">
-        <v>-8.741099999999999</v>
+        <v>-8.8691</v>
       </c>
       <c r="AG10" t="n">
-        <v>-6.1174</v>
-      </c>
+        <v>-6.045</v>
+      </c>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1969,7 +2029,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Credit to the non-government sector (excl. public corporations), percent of GDP</t>
+          <t>Credit to the non-government sector (claims on other sectors), percent of GDP</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1979,12 +2039,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1993,79 +2053,79 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>34.9781</v>
+        <v>37.4382</v>
       </c>
       <c r="K11" t="n">
-        <v>28.7264</v>
+        <v>32.9472</v>
       </c>
       <c r="L11" t="n">
-        <v>29.7609</v>
+        <v>34.0091</v>
       </c>
       <c r="M11" t="n">
-        <v>30.011</v>
+        <v>34.2605</v>
       </c>
       <c r="N11" t="n">
-        <v>33.6428</v>
+        <v>37.7881</v>
       </c>
       <c r="O11" t="n">
-        <v>37.3819</v>
+        <v>41.587</v>
       </c>
       <c r="P11" t="n">
-        <v>43.616</v>
+        <v>53.2879</v>
       </c>
       <c r="Q11" t="n">
-        <v>41.7613</v>
+        <v>53.3199</v>
       </c>
       <c r="R11" t="n">
-        <v>57.3718</v>
+        <v>69.749</v>
       </c>
       <c r="S11" t="n">
-        <v>46.7239</v>
+        <v>62.044</v>
       </c>
       <c r="T11" t="n">
-        <v>39.753</v>
+        <v>57.4997</v>
       </c>
       <c r="U11" t="n">
-        <v>39.4083</v>
+        <v>64.68170000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>41.9274</v>
+        <v>67.9053</v>
       </c>
       <c r="W11" t="n">
-        <v>48.3905</v>
+        <v>71.40560000000001</v>
       </c>
       <c r="X11" t="n">
-        <v>73.70140000000001</v>
+        <v>101.5796</v>
       </c>
       <c r="Y11" t="n">
-        <v>83.4973</v>
+        <v>112.0641</v>
       </c>
       <c r="Z11" t="n">
-        <v>83.8614</v>
+        <v>112.669</v>
       </c>
       <c r="AA11" t="n">
-        <v>82.9782</v>
+        <v>108.3952</v>
       </c>
       <c r="AB11" t="n">
-        <v>103.087</v>
+        <v>132.1299</v>
       </c>
       <c r="AC11" t="n">
-        <v>141.873</v>
+        <v>182.9785</v>
       </c>
       <c r="AD11" t="n">
-        <v>125.9861</v>
+        <v>162.3094</v>
       </c>
       <c r="AE11" t="n">
-        <v>103.0212</v>
+        <v>133.2579</v>
       </c>
       <c r="AF11" t="n">
-        <v>117.491</v>
+        <v>150.7827</v>
       </c>
       <c r="AG11" t="n">
-        <v>121.2823</v>
+        <v>156.3238</v>
       </c>
       <c r="AH11" t="n">
-        <v>125.3069</v>
+        <v>160.0833</v>
       </c>
     </row>
     <row r="12">
@@ -2101,12 +2161,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2114,50 +2174,60 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
-        <v>48.1645</v>
+        <v>63.882</v>
       </c>
       <c r="U12" t="n">
-        <v>46.9413</v>
+        <v>66.5377</v>
       </c>
       <c r="V12" t="n">
-        <v>46.6633</v>
+        <v>69.3289</v>
       </c>
       <c r="W12" t="n">
-        <v>48.0741</v>
+        <v>72.28879999999999</v>
       </c>
       <c r="X12" t="n">
-        <v>55.2688</v>
+        <v>81.824</v>
       </c>
       <c r="Y12" t="n">
-        <v>63.1956</v>
+        <v>91.7242</v>
       </c>
       <c r="Z12" t="n">
-        <v>69.625</v>
+        <v>99.7531</v>
       </c>
       <c r="AA12" t="n">
-        <v>74.6408</v>
+        <v>105.337</v>
       </c>
       <c r="AB12" t="n">
-        <v>82.649</v>
+        <v>114.4812</v>
       </c>
       <c r="AC12" t="n">
-        <v>96.49339999999999</v>
+        <v>131.483</v>
       </c>
       <c r="AD12" t="n">
-        <v>105.2503</v>
+        <v>142.0111</v>
       </c>
       <c r="AE12" t="n">
-        <v>108.6794</v>
+        <v>145.8679</v>
       </c>
       <c r="AF12" t="n">
-        <v>113.8962</v>
+        <v>151.9155</v>
       </c>
       <c r="AG12" t="n">
-        <v>118.9016</v>
+        <v>157.8789</v>
       </c>
       <c r="AH12" t="n">
-        <v>123.7662</v>
+        <v>163.5021</v>
       </c>
     </row>
     <row r="13">
@@ -2193,12 +2263,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Credit = claims on other sectors minus claims on public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors less claims on public non-financial corporations) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2206,50 +2276,60 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
-        <v>-8.4115</v>
+        <v>-6.3823</v>
       </c>
       <c r="U13" t="n">
-        <v>-7.5331</v>
+        <v>-1.8559</v>
       </c>
       <c r="V13" t="n">
-        <v>-4.7358</v>
+        <v>-1.4235</v>
       </c>
       <c r="W13" t="n">
-        <v>0.3163</v>
+        <v>-0.8832</v>
       </c>
       <c r="X13" t="n">
-        <v>18.4326</v>
+        <v>19.7556</v>
       </c>
       <c r="Y13" t="n">
-        <v>20.3017</v>
+        <v>20.3399</v>
       </c>
       <c r="Z13" t="n">
-        <v>14.2365</v>
+        <v>12.9159</v>
       </c>
       <c r="AA13" t="n">
-        <v>8.337300000000001</v>
+        <v>3.0582</v>
       </c>
       <c r="AB13" t="n">
-        <v>20.438</v>
+        <v>17.6487</v>
       </c>
       <c r="AC13" t="n">
-        <v>45.3797</v>
+        <v>51.4955</v>
       </c>
       <c r="AD13" t="n">
-        <v>20.7358</v>
+        <v>20.2983</v>
       </c>
       <c r="AE13" t="n">
-        <v>-5.6582</v>
+        <v>-12.6101</v>
       </c>
       <c r="AF13" t="n">
-        <v>3.5948</v>
+        <v>-1.1328</v>
       </c>
       <c r="AG13" t="n">
-        <v>2.3807</v>
+        <v>-1.5551</v>
       </c>
       <c r="AH13" t="n">
-        <v>1.5407</v>
+        <v>-3.4187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Credit gap: trend from the series start, start-up decade flagged, 20-year minimum
- Verified: one-sided HP always used all data from the first observation; hiding the
  first 10 years changed nothing later (max diff 0.0); quarterly gaps match BIS-published
  gaps exactly for SAU, GBR, USA, CHN, DEU, TUR; Kuwait gaps move 1-4 pp with the start year
- Now: trend and gap shown from the first year, first 10 years shaded as start-up
  period; no trend/gap for series under 20 years (user data too)
- README quotes BCBS (2010, Annex 1, p. 19); recompute_credit_gaps.py recomputes gaps
  from stored ratios when the BIS/IMF APIs are down; build flag --credit-only

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Trend: one-sided Hodrick-Prescott filter, lambda 100,000 (annual data), reported from 10 years after the series start. Gap = ratio - trend, percentage points of GDP.</t>
+          <t>Trend: one-sided Hodrick-Prescott filter, lambda 100,000 (annual data), from the series start; the first 10 years are a start-up period (less reliable). Gap = ratio - trend, percentage points of GDP.</t>
         </is>
       </c>
     </row>
@@ -480,61 +480,68 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>USER-BUILT GAPS: RECOMMENDED DATA LENGTH. Use at least 20 years (80 quarters) of credit-to-GDP data where possible, and never less than 10 years. The first 10 years only start the one-sided HP trend and are not reported, so with 10-20 years of data the gap covers fewer than 10 years and should be read with caution.</t>
+          <t>DATA LENGTH RULE (this tool): a gap is computed only when at least 20 years (80 quarters) of credit-to-GDP data are available. The one-sided HP filter starts at the first observation and the trend is shown from there, but the first 10 years are a start-up period: the trend is still settling and is sensitive to the starting year (charts shade it). BIS publishes the gap only from year 11.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Why: Drehmann and Tsatsaronis (2014, p. 14 of the article PDF) 'validate the practical rule of thumb that suggests using the credit gap only when at least 10 years of data for the credit-to-GDP ratio are already available', but note that at the start of a series 'it can take 20 years for measurement differences to fully disappear' (p. 13) and that 'we need at least 20 years of data in order to properly assess the forecasting ability of the credit gap' (p. 10). Credit cycles are 'on average about four times longer than standard business cycles and crises tend to occur once every 20-25 years' (p. 12).</t>
+          <t>Basel guidance: BCBS (2010, Annex 1, p. 19) defines the trend as 'a one sided Hodrick-Prescott filter with a high smoothing parameter' where 'only information available at each point in time is used', lambda 400,000 on quarterly data; it sets no minimum data length.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Structural breaks: adjust the credit series for breaks first; after a large break 'it takes more than 20 years for such an effect of this magnitude to fully disappear' (Drehmann and Tsatsaronis, 2014, p. 15).</t>
+          <t>Why: Drehmann and Tsatsaronis (2014, p. 14 of the article PDF) 'validate the practical rule of thumb that suggests using the credit gap only when at least 10 years of data for the credit-to-GDP ratio are already available', but note that at the start of a series 'it can take 20 years for measurement differences to fully disappear' (p. 13) and that 'we need at least 20 years of data in order to properly assess the forecasting ability of the credit gap' (p. 10). Credit cycles are 'on average about four times longer than standard business cycles and crises tend to occur once every 20-25 years' (p. 12).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Quarterly data (preferred): ratio = credit at end of quarter / sum of GDP over the last 4 quarters x 100; one-sided HP trend with lambda 400,000 (BCBS, 2010, Annex 1; ESRB Recommendation ESRB/2014/1, Annex, Part II).</t>
+          <t>Structural breaks: adjust the credit series for breaks first; after a large break 'it takes more than 20 years for such an effect of this magnitude to fully disappear' (Drehmann and Tsatsaronis, 2014, p. 15).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
+          <t>Quarterly data (preferred): ratio = credit at end of quarter / sum of GDP over the last 4 quarters x 100; one-sided HP trend with lambda 400,000 (BCBS, 2010, Annex 1; ESRB Recommendation ESRB/2014/1, Annex, Part II).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Oil exporters: a ratio to non-oil GDP (user data) avoids oil-price swings in GDP; say that the GDP measure is user data.</t>
+          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>References: BCBS (2010), Guidance for national authorities operating the countercyclical capital buffer, Basel Committee on Banking Supervision, December, https://www.bis.org/publ/bcbs187.htm. Drehmann, M. and K. Tsatsaronis (2014), 'The credit-to-GDP gap and countercyclical capital buffers: questions and answers', BIS Quarterly Review, March, https://www.bis.org/publ/qtrpdf/r_qt1403g.htm. ESRB (2014), Recommendation of the European Systemic Risk Board on guidance for setting countercyclical buffer rates (ESRB/2014/1), OJ C 293, 2.9.2014, https://www.esrb.europa.eu/pub/pdf/recommendations/140630_ESRB_Recommendation.en.pdf. Ravn, M. and H. Uhlig (2002), 'On adjusting the Hodrick-Prescott filter for the frequency of observations', Review of Economics and Statistics 84(2).</t>
+          <t>Oil exporters: a ratio to non-oil GDP (user data) avoids oil-price swings in GDP; say that the GDP measure is user data.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cite the 'Citation' column (IMF; trend and gap are own calculations), not this workbook.</t>
+          <t>References: BCBS (2010), Guidance for national authorities operating the countercyclical capital buffer, Basel Committee on Banking Supervision, December, https://www.bis.org/publ/bcbs187.htm. Drehmann, M. and K. Tsatsaronis (2014), 'The credit-to-GDP gap and countercyclical capital buffers: questions and answers', BIS Quarterly Review, March, https://www.bis.org/publ/qtrpdf/r_qt1403g.htm. ESRB (2014), Recommendation of the European Systemic Risk Board on guidance for setting countercyclical buffer rates (ESRB/2014/1), OJ C 293, 2.9.2014, https://www.esrb.europa.eu/pub/pdf/recommendations/140630_ESRB_Recommendation.en.pdf. Ravn, M. and H. Uhlig (2002), 'On adjusting the Hodrick-Prescott filter for the frequency of observations', Review of Economics and Statistics 84(2).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>Cite the 'Citation' column (IMF; trend and gap are own calculations), not this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>To refresh: run m365-agent/build_data_file.py and re-upload.</t>
         </is>
@@ -667,7 +674,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -714,7 +721,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -761,7 +768,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -799,16 +806,16 @@
         <v>-16.1</v>
       </c>
       <c r="I5" t="n">
-        <v>4.2</v>
+        <v>15.2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1074,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1189,7 +1196,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1202,18 +1209,38 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>36.7017</v>
+      </c>
+      <c r="K3" t="n">
+        <v>38.7969</v>
+      </c>
+      <c r="L3" t="n">
+        <v>40.1111</v>
+      </c>
+      <c r="M3" t="n">
+        <v>41.573</v>
+      </c>
+      <c r="N3" t="n">
+        <v>47.1328</v>
+      </c>
+      <c r="O3" t="n">
+        <v>52.7911</v>
+      </c>
+      <c r="P3" t="n">
+        <v>61.1864</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>72.1707</v>
+      </c>
+      <c r="R3" t="n">
+        <v>87.3905</v>
+      </c>
+      <c r="S3" t="n">
+        <v>91.8633</v>
+      </c>
       <c r="T3" t="n">
-        <v>91.47920000000001</v>
+        <v>91.47929999999999</v>
       </c>
       <c r="U3" t="n">
         <v>90.30800000000001</v>
@@ -1291,7 +1318,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1304,18 +1331,38 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.1562</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-0.0706</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2.6691</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2.516</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5.4802</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>8.7387</v>
+      </c>
+      <c r="R4" t="n">
+        <v>15.199</v>
+      </c>
+      <c r="S4" t="n">
+        <v>-5.9611</v>
+      </c>
       <c r="T4" t="n">
-        <v>-16.08</v>
+        <v>-16.0801</v>
       </c>
       <c r="U4" t="n">
         <v>-17.2583</v>
@@ -1330,7 +1377,7 @@
         <v>-1.092</v>
       </c>
       <c r="Y4" t="n">
-        <v>-0.4806</v>
+        <v>-0.4807</v>
       </c>
       <c r="Z4" t="n">
         <v>-7.6553</v>
@@ -1342,10 +1389,10 @@
         <v>-11.436</v>
       </c>
       <c r="AC4" t="n">
-        <v>4.1788</v>
+        <v>4.1789</v>
       </c>
       <c r="AD4" t="n">
-        <v>-11.277</v>
+        <v>-11.2769</v>
       </c>
       <c r="AE4" t="n">
         <v>-22.9076</v>
@@ -1393,7 +1440,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1515,7 +1562,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1528,16 +1575,36 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>57.2779</v>
+      </c>
+      <c r="K6" t="n">
+        <v>59.6603</v>
+      </c>
+      <c r="L6" t="n">
+        <v>60.8346</v>
+      </c>
+      <c r="M6" t="n">
+        <v>59.2902</v>
+      </c>
+      <c r="N6" t="n">
+        <v>54.6733</v>
+      </c>
+      <c r="O6" t="n">
+        <v>54.0954</v>
+      </c>
+      <c r="P6" t="n">
+        <v>59.4642</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>61.6647</v>
+      </c>
+      <c r="R6" t="n">
+        <v>72.29340000000001</v>
+      </c>
+      <c r="S6" t="n">
+        <v>77.6893</v>
+      </c>
       <c r="T6" t="n">
         <v>76.1014</v>
       </c>
@@ -1566,10 +1633,10 @@
         <v>97.4653</v>
       </c>
       <c r="AC6" t="n">
-        <v>104.2959</v>
+        <v>104.296</v>
       </c>
       <c r="AD6" t="n">
-        <v>105.7906</v>
+        <v>105.7907</v>
       </c>
       <c r="AE6" t="n">
         <v>104.566</v>
@@ -1617,7 +1684,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1630,16 +1697,36 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-0.2416</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-1.3722</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-3.2681</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.7009</v>
+      </c>
+      <c r="P7" t="n">
+        <v>7.5081</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2.5717</v>
+      </c>
+      <c r="R7" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>5.5271</v>
+      </c>
       <c r="T7" t="n">
         <v>-9.697100000000001</v>
       </c>
@@ -1659,7 +1746,7 @@
         <v>21.2887</v>
       </c>
       <c r="Z7" t="n">
-        <v>8.9619</v>
+        <v>8.962</v>
       </c>
       <c r="AA7" t="n">
         <v>-2.2839</v>
@@ -1671,13 +1758,13 @@
         <v>18.4549</v>
       </c>
       <c r="AD7" t="n">
-        <v>-6.6373</v>
+        <v>-6.6374</v>
       </c>
       <c r="AE7" t="n">
         <v>-19.6785</v>
       </c>
       <c r="AF7" t="n">
-        <v>-9.143599999999999</v>
+        <v>-9.143700000000001</v>
       </c>
       <c r="AG7" t="n">
         <v>-4.1278</v>
@@ -1719,7 +1806,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1839,7 +1926,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1852,18 +1939,38 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>35.4823</v>
+      </c>
+      <c r="K9" t="n">
+        <v>34.489</v>
+      </c>
+      <c r="L9" t="n">
+        <v>33.0016</v>
+      </c>
+      <c r="M9" t="n">
+        <v>30.9794</v>
+      </c>
+      <c r="N9" t="n">
+        <v>28.3399</v>
+      </c>
+      <c r="O9" t="n">
+        <v>27.2632</v>
+      </c>
+      <c r="P9" t="n">
+        <v>29.7696</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>31.1881</v>
+      </c>
+      <c r="R9" t="n">
+        <v>36.4603</v>
+      </c>
+      <c r="S9" t="n">
+        <v>39.5146</v>
+      </c>
       <c r="T9" t="n">
-        <v>41.3218</v>
+        <v>41.3219</v>
       </c>
       <c r="U9" t="n">
         <v>42.9118</v>
@@ -1899,7 +2006,7 @@
         <v>82.15519999999999</v>
       </c>
       <c r="AF9" t="n">
-        <v>83.2869</v>
+        <v>83.2868</v>
       </c>
       <c r="AG9" t="n">
         <v>84.9081</v>
@@ -1939,7 +2046,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1952,16 +2059,36 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-0.0988</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-0.3139</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-0.6905</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.7927999999999999</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4.866</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.0184</v>
+      </c>
+      <c r="R10" t="n">
+        <v>9.1869</v>
+      </c>
+      <c r="S10" t="n">
+        <v>4.5006</v>
+      </c>
       <c r="T10" t="n">
         <v>1.6141</v>
       </c>
@@ -1981,7 +2108,7 @@
         <v>17.6044</v>
       </c>
       <c r="Z10" t="n">
-        <v>11.3732</v>
+        <v>11.3733</v>
       </c>
       <c r="AA10" t="n">
         <v>3.2319</v>
@@ -1993,7 +2120,7 @@
         <v>12.9662</v>
       </c>
       <c r="AD10" t="n">
-        <v>1.3559</v>
+        <v>1.3558</v>
       </c>
       <c r="AE10" t="n">
         <v>-13.7025</v>
@@ -2002,7 +2129,7 @@
         <v>-8.8691</v>
       </c>
       <c r="AG10" t="n">
-        <v>-6.045</v>
+        <v>-6.0449</v>
       </c>
       <c r="AH10" t="inlineStr"/>
     </row>
@@ -2039,7 +2166,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2161,7 +2288,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2174,16 +2301,36 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>37.4382</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32.9472</v>
+      </c>
+      <c r="L12" t="n">
+        <v>33.0836</v>
+      </c>
+      <c r="M12" t="n">
+        <v>33.3931</v>
+      </c>
+      <c r="N12" t="n">
+        <v>35.6913</v>
+      </c>
+      <c r="O12" t="n">
+        <v>38.8754</v>
+      </c>
+      <c r="P12" t="n">
+        <v>46.1108</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>50.5442</v>
+      </c>
+      <c r="R12" t="n">
+        <v>59.5715</v>
+      </c>
+      <c r="S12" t="n">
+        <v>63.0033</v>
+      </c>
       <c r="T12" t="n">
         <v>63.882</v>
       </c>
@@ -2263,7 +2410,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, from 10 years after the series start</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2276,24 +2423,44 @@
           <t>https://data.imf.org</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.9255</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="N13" t="n">
+        <v>2.0968</v>
+      </c>
+      <c r="O13" t="n">
+        <v>2.7116</v>
+      </c>
+      <c r="P13" t="n">
+        <v>7.1771</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>2.7757</v>
+      </c>
+      <c r="R13" t="n">
+        <v>10.1775</v>
+      </c>
+      <c r="S13" t="n">
+        <v>-0.9593</v>
+      </c>
       <c r="T13" t="n">
         <v>-6.3823</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.8559</v>
+        <v>-1.856</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.4235</v>
+        <v>-1.4236</v>
       </c>
       <c r="W13" t="n">
         <v>-0.8832</v>
@@ -2320,7 +2487,7 @@
         <v>20.2983</v>
       </c>
       <c r="AE13" t="n">
-        <v>-12.6101</v>
+        <v>-12.61</v>
       </c>
       <c r="AF13" t="n">
         <v>-1.1328</v>
@@ -2329,7 +2496,7 @@
         <v>-1.5551</v>
       </c>
       <c r="AH13" t="n">
-        <v>-3.4187</v>
+        <v>-3.4188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Annual HP lambda = 400,000 / 4^4 = 1,562.5 (Ravn-Uhlig frequency adjustment)
Replaces 100,000 for annual data everywhere (library, agents, workbooks, docs).
Annual gaps now track BIS quarterly gaps (yearly averages) within 0.4-0.9 pp on
average for SAU, GBR, USA, CHN, DEU, TUR, JPN, BRA (100,000: 0.8-12.9 pp).
Kuwait 2025 gap 2.7 -> 3.3 pp.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/IMF_MFS_credit_to_GDP.xlsx
+++ b/m365-agent/IMF_MFS_credit_to_GDP.xlsx
@@ -459,7 +459,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Trend: one-sided Hodrick-Prescott filter, lambda 100,000 (annual data), from the series start; the first 10 years are a start-up period (less reliable). Gap = ratio - trend, percentage points of GDP.</t>
+          <t>Trend: one-sided Hodrick-Prescott filter, lambda 1,562.5 (annual data), from the series start; the first 10 years are a start-up period (less reliable). Gap = ratio - trend, percentage points of GDP.</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Annual data: this tool uses lambda 100,000, a project convention. The Basel guide is defined on quarterly data; frequency-adjustment rules (Ravn and Uhlig, 2002) would give a much smaller annual lambda (400,000 / 4^4 = about 1,600), so annual gaps are not directly comparable with BIS quarterly gaps.</t>
+          <t>Annual data: lambda 1,562.5 = 400,000 / 4^4, the Basel quarterly lambda adjusted for the frequency of observations (Ravn and Uhlig, 2002), so annual trends are about as smooth as BIS quarterly trends. The Basel guide itself is defined on quarterly data; prefer quarterly data when available.</t>
         </is>
       </c>
     </row>
@@ -649,23 +649,23 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -19.7, max 22.2</t>
+          <t>2014 to 2025: min -19.9, max 22.0</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>112.6</v>
       </c>
       <c r="F2" t="n">
-        <v>109.8</v>
+        <v>109.3</v>
       </c>
       <c r="G2" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="H2" t="n">
-        <v>-4.1</v>
+        <v>-3.5</v>
       </c>
       <c r="I2" t="n">
-        <v>22.2</v>
+        <v>22</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -691,28 +691,28 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>▄▅▇█▇▅▅▇▄▁▂▃</t>
+          <t>▅▅██▇▅▅▇▄▁▂▃</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2013 to 2024: min -13.7, max 17.6</t>
+          <t>2013 to 2024: min -14.9, max 16.8</t>
         </is>
       </c>
       <c r="E3" t="n">
         <v>78.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>84.90000000000001</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>-6</v>
+        <v>-6.2</v>
       </c>
       <c r="H3" t="n">
-        <v>-8.9</v>
+        <v>-9.5</v>
       </c>
       <c r="I3" t="n">
-        <v>17.6</v>
+        <v>16.8</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -738,28 +738,28 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>▂▅▅▄▃▄█▅▁▂▂▂</t>
+          <t>▃▅▅▄▃▅█▅▁▂▂▂</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -12.6, max 51.5</t>
+          <t>2014 to 2025: min -16.6, max 47.7</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>160.1</v>
       </c>
       <c r="F4" t="n">
-        <v>163.5</v>
+        <v>166.6</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.4</v>
+        <v>-6.6</v>
       </c>
       <c r="H4" t="n">
-        <v>-1.6</v>
+        <v>-5.1</v>
       </c>
       <c r="I4" t="n">
-        <v>51.5</v>
+        <v>47.7</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -768,7 +768,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -785,28 +785,28 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>▄▇▇▅▄▄█▄▁▂▃▄</t>
+          <t>▃▆▇▅▃▄█▄▁▃▃▅</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2014 to 2025: min -22.9, max 4.2</t>
+          <t>2014 to 2025: min -20.0, max 5.6</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>91.2</v>
       </c>
       <c r="F5" t="n">
-        <v>102.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>-11</v>
+        <v>-5.9</v>
       </c>
       <c r="H5" t="n">
-        <v>-16.1</v>
+        <v>-11.5</v>
       </c>
       <c r="I5" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
     <col width="9" customWidth="1" min="24" max="24"/>
     <col width="9" customWidth="1" min="25" max="25"/>
     <col width="9" customWidth="1" min="26" max="26"/>
-    <col width="9" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
     <col width="9" customWidth="1" min="28" max="28"/>
     <col width="10" customWidth="1" min="29" max="29"/>
     <col width="10" customWidth="1" min="30" max="30"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1196,12 +1196,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1222,67 +1222,67 @@
         <v>41.573</v>
       </c>
       <c r="N3" t="n">
-        <v>47.1328</v>
+        <v>47.1342</v>
       </c>
       <c r="O3" t="n">
-        <v>52.7911</v>
+        <v>52.7955</v>
       </c>
       <c r="P3" t="n">
-        <v>61.1864</v>
+        <v>61.2005</v>
       </c>
       <c r="Q3" t="n">
-        <v>72.1707</v>
+        <v>72.2089</v>
       </c>
       <c r="R3" t="n">
-        <v>87.3905</v>
+        <v>87.48909999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>91.8633</v>
+        <v>91.94110000000001</v>
       </c>
       <c r="T3" t="n">
-        <v>91.47929999999999</v>
+        <v>91.447</v>
       </c>
       <c r="U3" t="n">
-        <v>90.30800000000001</v>
+        <v>90.10760000000001</v>
       </c>
       <c r="V3" t="n">
-        <v>89.8339</v>
+        <v>89.4409</v>
       </c>
       <c r="W3" t="n">
-        <v>89.7681</v>
+        <v>89.1609</v>
       </c>
       <c r="X3" t="n">
-        <v>93.35429999999999</v>
+        <v>92.6979</v>
       </c>
       <c r="Y3" t="n">
-        <v>97.11069999999999</v>
+        <v>96.4306</v>
       </c>
       <c r="Z3" t="n">
-        <v>98.886</v>
+        <v>98.0172</v>
       </c>
       <c r="AA3" t="n">
-        <v>99.20010000000001</v>
+        <v>97.9558</v>
       </c>
       <c r="AB3" t="n">
-        <v>99.8267</v>
+        <v>98.2022</v>
       </c>
       <c r="AC3" t="n">
-        <v>103.9576</v>
+        <v>102.4993</v>
       </c>
       <c r="AD3" t="n">
-        <v>104.7614</v>
+        <v>102.8652</v>
       </c>
       <c r="AE3" t="n">
-        <v>103.1124</v>
+        <v>100.1803</v>
       </c>
       <c r="AF3" t="n">
-        <v>102.4087</v>
+        <v>98.6198</v>
       </c>
       <c r="AG3" t="n">
-        <v>101.8875</v>
+        <v>97.2748</v>
       </c>
       <c r="AH3" t="n">
-        <v>102.2213</v>
+        <v>97.0817</v>
       </c>
     </row>
     <row r="4">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1344,67 +1344,67 @@
         <v>-0.0706</v>
       </c>
       <c r="N4" t="n">
-        <v>2.6691</v>
+        <v>2.6677</v>
       </c>
       <c r="O4" t="n">
-        <v>2.516</v>
+        <v>2.5116</v>
       </c>
       <c r="P4" t="n">
-        <v>5.4802</v>
+        <v>5.4661</v>
       </c>
       <c r="Q4" t="n">
-        <v>8.7387</v>
+        <v>8.7005</v>
       </c>
       <c r="R4" t="n">
-        <v>15.199</v>
+        <v>15.1004</v>
       </c>
       <c r="S4" t="n">
-        <v>-5.9611</v>
+        <v>-6.0389</v>
       </c>
       <c r="T4" t="n">
-        <v>-16.0801</v>
+        <v>-16.0478</v>
       </c>
       <c r="U4" t="n">
-        <v>-17.2583</v>
+        <v>-17.0579</v>
       </c>
       <c r="V4" t="n">
-        <v>-14.7228</v>
+        <v>-14.3298</v>
       </c>
       <c r="W4" t="n">
-        <v>-12.9929</v>
+        <v>-12.3857</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.092</v>
+        <v>-0.4356</v>
       </c>
       <c r="Y4" t="n">
-        <v>-0.4807</v>
+        <v>0.1994</v>
       </c>
       <c r="Z4" t="n">
-        <v>-7.6553</v>
+        <v>-6.7865</v>
       </c>
       <c r="AA4" t="n">
-        <v>-13.0931</v>
+        <v>-11.8488</v>
       </c>
       <c r="AB4" t="n">
-        <v>-11.436</v>
+        <v>-9.811500000000001</v>
       </c>
       <c r="AC4" t="n">
-        <v>4.1789</v>
+        <v>5.6372</v>
       </c>
       <c r="AD4" t="n">
-        <v>-11.2769</v>
+        <v>-9.380699999999999</v>
       </c>
       <c r="AE4" t="n">
-        <v>-22.9076</v>
+        <v>-19.9755</v>
       </c>
       <c r="AF4" t="n">
-        <v>-17.5311</v>
+        <v>-13.7422</v>
       </c>
       <c r="AG4" t="n">
-        <v>-16.1431</v>
+        <v>-11.5304</v>
       </c>
       <c r="AH4" t="n">
-        <v>-10.9997</v>
+        <v>-5.8601</v>
       </c>
     </row>
     <row r="5">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1585,70 +1585,70 @@
         <v>60.8346</v>
       </c>
       <c r="M6" t="n">
-        <v>59.2902</v>
+        <v>59.2898</v>
       </c>
       <c r="N6" t="n">
-        <v>54.6733</v>
+        <v>54.671</v>
       </c>
       <c r="O6" t="n">
-        <v>54.0954</v>
+        <v>54.0934</v>
       </c>
       <c r="P6" t="n">
-        <v>59.4642</v>
+        <v>59.4748</v>
       </c>
       <c r="Q6" t="n">
-        <v>61.6647</v>
+        <v>61.684</v>
       </c>
       <c r="R6" t="n">
-        <v>72.29340000000001</v>
+        <v>72.3751</v>
       </c>
       <c r="S6" t="n">
-        <v>77.6893</v>
+        <v>77.8087</v>
       </c>
       <c r="T6" t="n">
-        <v>76.1014</v>
+        <v>76.1622</v>
       </c>
       <c r="U6" t="n">
-        <v>72.8361</v>
+        <v>72.77370000000001</v>
       </c>
       <c r="V6" t="n">
-        <v>71.27249999999999</v>
+        <v>71.09990000000001</v>
       </c>
       <c r="W6" t="n">
-        <v>71.9992</v>
+        <v>71.7885</v>
       </c>
       <c r="X6" t="n">
-        <v>80.217</v>
+        <v>80.37869999999999</v>
       </c>
       <c r="Y6" t="n">
-        <v>88.3849</v>
+        <v>89.01260000000001</v>
       </c>
       <c r="Z6" t="n">
-        <v>93.3385</v>
+        <v>94.22929999999999</v>
       </c>
       <c r="AA6" t="n">
-        <v>95.459</v>
+        <v>96.3167</v>
       </c>
       <c r="AB6" t="n">
-        <v>97.4653</v>
+        <v>98.23950000000001</v>
       </c>
       <c r="AC6" t="n">
-        <v>104.296</v>
+        <v>105.7529</v>
       </c>
       <c r="AD6" t="n">
-        <v>105.7907</v>
+        <v>106.9601</v>
       </c>
       <c r="AE6" t="n">
-        <v>104.566</v>
+        <v>104.7634</v>
       </c>
       <c r="AF6" t="n">
-        <v>105.3136</v>
+        <v>104.9646</v>
       </c>
       <c r="AG6" t="n">
-        <v>106.96</v>
+        <v>106.314</v>
       </c>
       <c r="AH6" t="n">
-        <v>109.8197</v>
+        <v>109.3035</v>
       </c>
     </row>
     <row r="7">
@@ -1684,12 +1684,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1707,70 +1707,70 @@
         <v>-0.2416</v>
       </c>
       <c r="M7" t="n">
-        <v>-1.3722</v>
+        <v>-1.3718</v>
       </c>
       <c r="N7" t="n">
-        <v>-3.2681</v>
+        <v>-3.2658</v>
       </c>
       <c r="O7" t="n">
-        <v>0.7009</v>
+        <v>0.7029</v>
       </c>
       <c r="P7" t="n">
-        <v>7.5081</v>
+        <v>7.4975</v>
       </c>
       <c r="Q7" t="n">
-        <v>2.5717</v>
+        <v>2.5524</v>
       </c>
       <c r="R7" t="n">
-        <v>16.3</v>
+        <v>16.2183</v>
       </c>
       <c r="S7" t="n">
-        <v>5.5271</v>
+        <v>5.4077</v>
       </c>
       <c r="T7" t="n">
-        <v>-9.697100000000001</v>
+        <v>-9.757899999999999</v>
       </c>
       <c r="U7" t="n">
-        <v>-13.2822</v>
+        <v>-13.2198</v>
       </c>
       <c r="V7" t="n">
-        <v>-8.2569</v>
+        <v>-8.084300000000001</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.3372</v>
+        <v>-1.1265</v>
       </c>
       <c r="X7" t="n">
-        <v>22.1878</v>
+        <v>22.0261</v>
       </c>
       <c r="Y7" t="n">
-        <v>21.2887</v>
+        <v>20.661</v>
       </c>
       <c r="Z7" t="n">
-        <v>8.962</v>
+        <v>8.071199999999999</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.2839</v>
+        <v>-3.1416</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.6906</v>
+        <v>-3.4648</v>
       </c>
       <c r="AC7" t="n">
-        <v>18.4549</v>
+        <v>16.998</v>
       </c>
       <c r="AD7" t="n">
-        <v>-6.6374</v>
+        <v>-7.8068</v>
       </c>
       <c r="AE7" t="n">
-        <v>-19.6785</v>
+        <v>-19.8759</v>
       </c>
       <c r="AF7" t="n">
-        <v>-9.143700000000001</v>
+        <v>-8.794700000000001</v>
       </c>
       <c r="AG7" t="n">
-        <v>-4.1278</v>
+        <v>-3.4818</v>
       </c>
       <c r="AH7" t="n">
-        <v>2.7393</v>
+        <v>3.2555</v>
       </c>
     </row>
     <row r="8">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1926,12 +1926,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1949,67 +1949,67 @@
         <v>33.0016</v>
       </c>
       <c r="M9" t="n">
-        <v>30.9794</v>
+        <v>30.9793</v>
       </c>
       <c r="N9" t="n">
-        <v>28.3399</v>
+        <v>28.3394</v>
       </c>
       <c r="O9" t="n">
-        <v>27.2632</v>
+        <v>27.2634</v>
       </c>
       <c r="P9" t="n">
-        <v>29.7696</v>
+        <v>29.778</v>
       </c>
       <c r="Q9" t="n">
-        <v>31.1881</v>
+        <v>31.2058</v>
       </c>
       <c r="R9" t="n">
-        <v>36.4603</v>
+        <v>36.5138</v>
       </c>
       <c r="S9" t="n">
-        <v>39.5146</v>
+        <v>39.5967</v>
       </c>
       <c r="T9" t="n">
-        <v>41.3219</v>
+        <v>41.4206</v>
       </c>
       <c r="U9" t="n">
-        <v>42.9118</v>
+        <v>43.0234</v>
       </c>
       <c r="V9" t="n">
-        <v>44.5879</v>
+        <v>44.715</v>
       </c>
       <c r="W9" t="n">
-        <v>46.7672</v>
+        <v>46.9321</v>
       </c>
       <c r="X9" t="n">
-        <v>52.9337</v>
+        <v>53.3607</v>
       </c>
       <c r="Y9" t="n">
-        <v>60.01</v>
+        <v>60.8213</v>
       </c>
       <c r="Z9" t="n">
-        <v>65.5201</v>
+        <v>66.64109999999999</v>
       </c>
       <c r="AA9" t="n">
-        <v>69.0164</v>
+        <v>70.2535</v>
       </c>
       <c r="AB9" t="n">
-        <v>72.777</v>
+        <v>74.1561</v>
       </c>
       <c r="AC9" t="n">
-        <v>78.5637</v>
+        <v>80.4166</v>
       </c>
       <c r="AD9" t="n">
-        <v>81.9062</v>
+        <v>83.7928</v>
       </c>
       <c r="AE9" t="n">
-        <v>82.15519999999999</v>
+        <v>83.3385</v>
       </c>
       <c r="AF9" t="n">
-        <v>83.2868</v>
+        <v>83.9166</v>
       </c>
       <c r="AG9" t="n">
-        <v>84.9081</v>
+        <v>85.09439999999999</v>
       </c>
       <c r="AH9" t="inlineStr"/>
     </row>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2069,67 +2069,67 @@
         <v>-0.0988</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.3139</v>
+        <v>-0.3138</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.6905</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="O10" t="n">
-        <v>0.7927999999999999</v>
+        <v>0.7926</v>
       </c>
       <c r="P10" t="n">
-        <v>4.866</v>
+        <v>4.8576</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.0184</v>
+        <v>3.0007</v>
       </c>
       <c r="R10" t="n">
-        <v>9.1869</v>
+        <v>9.1334</v>
       </c>
       <c r="S10" t="n">
-        <v>4.5006</v>
+        <v>4.4185</v>
       </c>
       <c r="T10" t="n">
-        <v>1.6141</v>
+        <v>1.5154</v>
       </c>
       <c r="U10" t="n">
-        <v>1.0243</v>
+        <v>0.9127</v>
       </c>
       <c r="V10" t="n">
-        <v>1.21</v>
+        <v>1.0829</v>
       </c>
       <c r="W10" t="n">
-        <v>2.6172</v>
+        <v>2.4523</v>
       </c>
       <c r="X10" t="n">
-        <v>15.0221</v>
+        <v>14.5951</v>
       </c>
       <c r="Y10" t="n">
-        <v>17.6044</v>
+        <v>16.7931</v>
       </c>
       <c r="Z10" t="n">
-        <v>11.3733</v>
+        <v>10.2523</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.2319</v>
+        <v>1.9948</v>
       </c>
       <c r="AB10" t="n">
-        <v>4.2303</v>
+        <v>2.8512</v>
       </c>
       <c r="AC10" t="n">
-        <v>12.9662</v>
+        <v>11.1133</v>
       </c>
       <c r="AD10" t="n">
-        <v>1.3558</v>
+        <v>-0.5308</v>
       </c>
       <c r="AE10" t="n">
-        <v>-13.7025</v>
+        <v>-14.8858</v>
       </c>
       <c r="AF10" t="n">
-        <v>-8.8691</v>
+        <v>-9.498900000000001</v>
       </c>
       <c r="AG10" t="n">
-        <v>-6.0449</v>
+        <v>-6.2312</v>
       </c>
       <c r="AH10" t="inlineStr"/>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2288,12 +2288,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); trend: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2308,73 +2308,73 @@
         <v>32.9472</v>
       </c>
       <c r="L12" t="n">
-        <v>33.0836</v>
+        <v>33.0837</v>
       </c>
       <c r="M12" t="n">
-        <v>33.3931</v>
+        <v>33.3934</v>
       </c>
       <c r="N12" t="n">
-        <v>35.6913</v>
+        <v>35.6929</v>
       </c>
       <c r="O12" t="n">
-        <v>38.8754</v>
+        <v>38.8801</v>
       </c>
       <c r="P12" t="n">
-        <v>46.1108</v>
+        <v>46.1281</v>
       </c>
       <c r="Q12" t="n">
-        <v>50.5442</v>
+        <v>50.5708</v>
       </c>
       <c r="R12" t="n">
-        <v>59.5715</v>
+        <v>59.6378</v>
       </c>
       <c r="S12" t="n">
-        <v>63.0033</v>
+        <v>63.0706</v>
       </c>
       <c r="T12" t="n">
-        <v>63.882</v>
+        <v>63.9075</v>
       </c>
       <c r="U12" t="n">
-        <v>66.5377</v>
+        <v>66.54170000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>69.3289</v>
+        <v>69.3112</v>
       </c>
       <c r="W12" t="n">
-        <v>72.28879999999999</v>
+        <v>72.2531</v>
       </c>
       <c r="X12" t="n">
-        <v>81.824</v>
+        <v>82.1264</v>
       </c>
       <c r="Y12" t="n">
-        <v>91.7242</v>
+        <v>92.4727</v>
       </c>
       <c r="Z12" t="n">
-        <v>99.7531</v>
+        <v>100.8585</v>
       </c>
       <c r="AA12" t="n">
-        <v>105.337</v>
+        <v>106.5637</v>
       </c>
       <c r="AB12" t="n">
-        <v>114.4812</v>
+        <v>116.3032</v>
       </c>
       <c r="AC12" t="n">
-        <v>131.483</v>
+        <v>135.2584</v>
       </c>
       <c r="AD12" t="n">
-        <v>142.0111</v>
+        <v>146.6796</v>
       </c>
       <c r="AE12" t="n">
-        <v>145.8679</v>
+        <v>149.9065</v>
       </c>
       <c r="AF12" t="n">
-        <v>151.9155</v>
+        <v>155.7665</v>
       </c>
       <c r="AG12" t="n">
-        <v>157.8789</v>
+        <v>161.4577</v>
       </c>
       <c r="AH12" t="n">
-        <v>163.5021</v>
+        <v>166.6454</v>
       </c>
     </row>
     <row r="13">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 100,000, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
+          <t>Credit = depository corporations' claims on other sectors, incl. public non-financial corporations (end of year); ratio = credit / nominal GDP x 100; trend: one-sided HP filter, lambda = 1,562.5, trend from the series start (first 10 years = start-up period); no gap for series under 20 years</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 100,000)</t>
+          <t>International Monetary Fund, Monetary and Financial Statistics (dataset IMF.STA:MFS_DC; depository corporations' claims on other sectors) and World Economic Outlook (nominal GDP); gap: own calculation, one-sided HP filter (lambda 1,562.5)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2430,73 +2430,73 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0.9255</v>
+        <v>0.9254</v>
       </c>
       <c r="M13" t="n">
-        <v>0.8673999999999999</v>
+        <v>0.8671</v>
       </c>
       <c r="N13" t="n">
-        <v>2.0968</v>
+        <v>2.0952</v>
       </c>
       <c r="O13" t="n">
-        <v>2.7116</v>
+        <v>2.7069</v>
       </c>
       <c r="P13" t="n">
-        <v>7.1771</v>
+        <v>7.1598</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.7757</v>
+        <v>2.7491</v>
       </c>
       <c r="R13" t="n">
-        <v>10.1775</v>
+        <v>10.1112</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.9593</v>
+        <v>-1.0266</v>
       </c>
       <c r="T13" t="n">
-        <v>-6.3823</v>
+        <v>-6.4078</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.856</v>
+        <v>-1.86</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.4236</v>
+        <v>-1.4059</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.8832</v>
+        <v>-0.8475</v>
       </c>
       <c r="X13" t="n">
-        <v>19.7556</v>
+        <v>19.4532</v>
       </c>
       <c r="Y13" t="n">
-        <v>20.3399</v>
+        <v>19.5914</v>
       </c>
       <c r="Z13" t="n">
-        <v>12.9159</v>
+        <v>11.8105</v>
       </c>
       <c r="AA13" t="n">
-        <v>3.0582</v>
+        <v>1.8315</v>
       </c>
       <c r="AB13" t="n">
-        <v>17.6487</v>
+        <v>15.8267</v>
       </c>
       <c r="AC13" t="n">
-        <v>51.4955</v>
+        <v>47.7201</v>
       </c>
       <c r="AD13" t="n">
-        <v>20.2983</v>
+        <v>15.6298</v>
       </c>
       <c r="AE13" t="n">
-        <v>-12.61</v>
+        <v>-16.6486</v>
       </c>
       <c r="AF13" t="n">
-        <v>-1.1328</v>
+        <v>-4.9838</v>
       </c>
       <c r="AG13" t="n">
-        <v>-1.5551</v>
+        <v>-5.1339</v>
       </c>
       <c r="AH13" t="n">
-        <v>-3.4188</v>
+        <v>-6.5621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>